<commit_message>
clean parameters for paper0
</commit_message>
<xml_diff>
--- a/scenarios/Coal_Flexibilisation/sub_scenarios/reserve_margin.xlsx
+++ b/scenarios/Coal_Flexibilisation/sub_scenarios/reserve_margin.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Meridian Dropbox\ME Projects\01 PROJECTS &amp; PROPOSALS\PyPSA scenarios\Coal flex\sub_scenarios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agatha.majcher\Downloads\agma0 pypsa-rsa master scenarios-Coal_Flexibilisation\sub_scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E915201-9E81-43C8-8FE5-95CBDC9392DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00CF55D6-C72A-4742-BACA-D85AC4DC6CF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="450" yWindow="-15030" windowWidth="28455" windowHeight="12165" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="reserve_margin" sheetId="2" r:id="rId1"/>
     <sheet name="capacity_credits" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="41">
   <si>
     <t>technology</t>
   </si>
@@ -226,7 +226,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -295,6 +295,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -369,7 +375,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
@@ -418,13 +424,17 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="12" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="1" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
+    <cellStyle name="Ausgabe" xfId="4" builtinId="21"/>
     <cellStyle name="Excel Built-in Heading 2" xfId="2" xr:uid="{1E9D77BB-93FA-4263-AFE4-2945AE6ACE30}"/>
     <cellStyle name="Excel Built-in Input" xfId="3" xr:uid="{37DB297F-BE65-46B1-9561-536EF022F687}"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Output" xfId="4" builtinId="21"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Prozent" xfId="1" builtinId="5"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -717,20 +727,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF20C7E1-769F-4B9F-859A-2E4C5E6D79B9}">
-  <dimension ref="A1:AU9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AC9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
     <col min="2" max="2" width="27.42578125" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" style="19" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" customWidth="1"/>
-    <col min="6" max="8" width="7.42578125" customWidth="1"/>
-    <col min="9" max="36" width="9.42578125" style="4" customWidth="1"/>
-    <col min="37" max="37" width="7.85546875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" style="4" customWidth="1"/>
+    <col min="5" max="28" width="9.42578125" style="4" customWidth="1"/>
+    <col min="29" max="29" width="7.85546875" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>28</v>
       </c>
@@ -741,149 +749,85 @@
         <v>39</v>
       </c>
       <c r="D1" s="5">
-        <v>2017</v>
+        <v>2025</v>
       </c>
       <c r="E1" s="5">
-        <v>2018</v>
+        <v>2026</v>
       </c>
       <c r="F1" s="5">
-        <v>2019</v>
+        <v>2027</v>
       </c>
       <c r="G1" s="5">
-        <v>2020</v>
+        <v>2028</v>
       </c>
       <c r="H1" s="5">
-        <v>2021</v>
+        <v>2029</v>
       </c>
       <c r="I1" s="5">
-        <v>2022</v>
+        <v>2030</v>
       </c>
       <c r="J1" s="5">
-        <v>2023</v>
+        <v>2031</v>
       </c>
       <c r="K1" s="5">
-        <v>2024</v>
+        <v>2032</v>
       </c>
       <c r="L1" s="5">
-        <v>2025</v>
+        <v>2033</v>
       </c>
       <c r="M1" s="5">
-        <v>2026</v>
+        <v>2034</v>
       </c>
       <c r="N1" s="5">
-        <v>2027</v>
+        <v>2035</v>
       </c>
       <c r="O1" s="5">
-        <v>2028</v>
+        <v>2036</v>
       </c>
       <c r="P1" s="5">
-        <v>2029</v>
+        <v>2037</v>
       </c>
       <c r="Q1" s="5">
-        <v>2030</v>
+        <v>2038</v>
       </c>
       <c r="R1" s="5">
-        <v>2031</v>
+        <v>2039</v>
       </c>
       <c r="S1" s="5">
-        <v>2032</v>
+        <v>2040</v>
       </c>
       <c r="T1" s="5">
-        <v>2033</v>
+        <v>2041</v>
       </c>
       <c r="U1" s="5">
-        <v>2034</v>
+        <v>2042</v>
       </c>
       <c r="V1" s="5">
-        <v>2035</v>
+        <v>2043</v>
       </c>
       <c r="W1" s="5">
-        <v>2036</v>
+        <v>2044</v>
       </c>
       <c r="X1" s="5">
-        <v>2037</v>
+        <v>2045</v>
       </c>
       <c r="Y1" s="5">
-        <v>2038</v>
+        <v>2046</v>
       </c>
       <c r="Z1" s="5">
-        <v>2039</v>
+        <v>2047</v>
       </c>
       <c r="AA1" s="5">
-        <v>2040</v>
+        <v>2048</v>
       </c>
       <c r="AB1" s="5">
-        <v>2041</v>
+        <v>2049</v>
       </c>
       <c r="AC1" s="5">
-        <v>2042</v>
-      </c>
-      <c r="AD1" s="5">
-        <v>2043</v>
-      </c>
-      <c r="AE1" s="5">
-        <v>2044</v>
-      </c>
-      <c r="AF1" s="5">
-        <v>2045</v>
-      </c>
-      <c r="AG1" s="5">
-        <v>2046</v>
-      </c>
-      <c r="AH1" s="5">
-        <v>2047</v>
-      </c>
-      <c r="AI1" s="5">
-        <v>2048</v>
-      </c>
-      <c r="AJ1" s="5">
-        <v>2049</v>
-      </c>
-      <c r="AK1" s="5">
         <v>2050</v>
       </c>
-      <c r="AL1" s="5">
-        <f t="shared" ref="AL1:AU1" si="0">AK1+1</f>
-        <v>2051</v>
-      </c>
-      <c r="AM1" s="5">
-        <f t="shared" si="0"/>
-        <v>2052</v>
-      </c>
-      <c r="AN1" s="5">
-        <f t="shared" si="0"/>
-        <v>2053</v>
-      </c>
-      <c r="AO1" s="5">
-        <f t="shared" si="0"/>
-        <v>2054</v>
-      </c>
-      <c r="AP1" s="5">
-        <f t="shared" si="0"/>
-        <v>2055</v>
-      </c>
-      <c r="AQ1" s="5">
-        <f t="shared" si="0"/>
-        <v>2056</v>
-      </c>
-      <c r="AR1" s="5">
-        <f t="shared" si="0"/>
-        <v>2057</v>
-      </c>
-      <c r="AS1" s="5">
-        <f t="shared" si="0"/>
-        <v>2058</v>
-      </c>
-      <c r="AT1" s="5">
-        <f t="shared" si="0"/>
-        <v>2059</v>
-      </c>
-      <c r="AU1" s="5">
-        <f t="shared" si="0"/>
-        <v>2060</v>
-      </c>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
@@ -894,186 +838,87 @@
         <v>32</v>
       </c>
       <c r="D2" s="8" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="E2" s="8" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="F2" s="8" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="G2" s="8" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="H2" s="8" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="I2" s="8" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="J2" s="8" t="b">
-        <f t="shared" ref="J2:Y8" si="1">I2</f>
         <v>0</v>
       </c>
       <c r="K2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="S2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="T2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="U2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="V2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="W2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="X2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y2" s="8" t="b">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z2" s="8" t="b">
-        <f t="shared" ref="Z2:AK8" si="2">Y2</f>
         <v>0</v>
       </c>
       <c r="AA2" s="8" t="b">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AB2" s="8" t="b">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AC2" s="8" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AD2" s="8" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AE2" s="8" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AF2" s="8" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AG2" s="8" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AH2" s="8" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AI2" s="8" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AJ2" s="8" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AK2" s="8" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AL2" s="8" t="b">
-        <f>AK2</f>
-        <v>0</v>
-      </c>
-      <c r="AM2" s="8" t="b">
-        <f t="shared" ref="AM2:AU2" si="3">AL2</f>
-        <v>0</v>
-      </c>
-      <c r="AN2" s="8" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AO2" s="8" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AP2" s="8" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AQ2" s="8" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AR2" s="8" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AS2" s="8" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AT2" s="8" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AU2" s="8" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="str">
-        <f>A2</f>
-        <v>RES_MRGN_0</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>33</v>
@@ -1159,72 +1004,8 @@
       <c r="AC3" s="11">
         <v>0</v>
       </c>
-      <c r="AD3" s="11">
-        <v>0</v>
-      </c>
-      <c r="AE3" s="11">
-        <v>0</v>
-      </c>
-      <c r="AF3" s="11">
-        <v>0</v>
-      </c>
-      <c r="AG3" s="11">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="11">
-        <v>0</v>
-      </c>
-      <c r="AI3" s="11">
-        <v>0</v>
-      </c>
-      <c r="AJ3" s="11">
-        <v>0</v>
-      </c>
-      <c r="AK3" s="11">
-        <v>0</v>
-      </c>
-      <c r="AL3" s="8">
-        <f t="shared" ref="AL3:AU3" si="4">AK3</f>
-        <v>0</v>
-      </c>
-      <c r="AM3" s="8">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AN3" s="8">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AO3" s="8">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AP3" s="8">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AQ3" s="8">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AR3" s="8">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AS3" s="8">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AT3" s="8">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AU3" s="8">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -1235,186 +1016,87 @@
         <v>32</v>
       </c>
       <c r="D4" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="E4" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="F4" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="G4" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="H4" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="I4" s="10" t="b">
-        <f>FALSE()</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" s="10" t="b">
-        <f t="shared" ref="J4:R5" si="5">I4</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" s="10" t="b">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L4" s="10" t="b">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" s="10" t="b">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" s="10" t="b">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4" s="10" t="b">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P4" s="10" t="b">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q4" s="10" t="b">
-        <f>TRUE()</f>
         <v>1</v>
       </c>
       <c r="R4" s="10" t="b">
-        <f>TRUE()</f>
         <v>1</v>
       </c>
       <c r="S4" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="T4" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="U4" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="V4" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="W4" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="X4" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="Y4" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="Z4" s="10" t="b">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="AA4" s="10" t="b">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="AB4" s="10" t="b">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="AC4" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AD4" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AE4" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AF4" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AG4" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AH4" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AI4" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AJ4" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AK4" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AL4" s="8" t="b">
-        <f t="shared" ref="AL4:AU4" si="6">AK4</f>
-        <v>1</v>
-      </c>
-      <c r="AM4" s="8" t="b">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
-      <c r="AN4" s="8" t="b">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
-      <c r="AO4" s="8" t="b">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
-      <c r="AP4" s="8" t="b">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
-      <c r="AQ4" s="8" t="b">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
-      <c r="AR4" s="8" t="b">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
-      <c r="AS4" s="8" t="b">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
-      <c r="AT4" s="8" t="b">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
-      <c r="AU4" s="8" t="b">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="str">
-        <f>A4</f>
-        <v>RES_MRGN_5</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>33</v>
@@ -1435,166 +1117,73 @@
         <v>0.05</v>
       </c>
       <c r="H5" s="11">
-        <f>G5</f>
         <v>0.05</v>
       </c>
       <c r="I5" s="11">
-        <f>H5</f>
         <v>0.05</v>
       </c>
       <c r="J5" s="11">
         <v>0.05</v>
       </c>
       <c r="K5" s="11">
-        <f t="shared" si="5"/>
         <v>0.05</v>
       </c>
       <c r="L5" s="11">
-        <f t="shared" si="5"/>
         <v>0.05</v>
       </c>
       <c r="M5" s="11">
-        <f t="shared" si="5"/>
         <v>0.05</v>
       </c>
       <c r="N5" s="11">
-        <f t="shared" si="5"/>
         <v>0.05</v>
       </c>
       <c r="O5" s="11">
-        <f t="shared" si="5"/>
         <v>0.05</v>
       </c>
       <c r="P5" s="11">
-        <f t="shared" si="5"/>
         <v>0.05</v>
       </c>
       <c r="Q5" s="11">
-        <f t="shared" si="5"/>
         <v>0.05</v>
       </c>
       <c r="R5" s="11">
-        <f t="shared" si="5"/>
         <v>0.05</v>
       </c>
       <c r="S5" s="11">
-        <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
       <c r="T5" s="11">
-        <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
       <c r="U5" s="11">
-        <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
       <c r="V5" s="11">
-        <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
       <c r="W5" s="11">
-        <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
       <c r="X5" s="11">
-        <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
       <c r="Y5" s="11">
-        <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
       <c r="Z5" s="11">
-        <f t="shared" si="2"/>
         <v>0.05</v>
       </c>
       <c r="AA5" s="11">
-        <f t="shared" si="2"/>
         <v>0.05</v>
       </c>
       <c r="AB5" s="11">
-        <f t="shared" si="2"/>
         <v>0.05</v>
       </c>
       <c r="AC5" s="11">
-        <f t="shared" si="2"/>
-        <v>0.05</v>
-      </c>
-      <c r="AD5" s="11">
-        <f t="shared" si="2"/>
-        <v>0.05</v>
-      </c>
-      <c r="AE5" s="11">
-        <f t="shared" si="2"/>
-        <v>0.05</v>
-      </c>
-      <c r="AF5" s="11">
-        <f t="shared" si="2"/>
-        <v>0.05</v>
-      </c>
-      <c r="AG5" s="11">
-        <f t="shared" si="2"/>
-        <v>0.05</v>
-      </c>
-      <c r="AH5" s="11">
-        <f t="shared" si="2"/>
-        <v>0.05</v>
-      </c>
-      <c r="AI5" s="11">
-        <f t="shared" si="2"/>
-        <v>0.05</v>
-      </c>
-      <c r="AJ5" s="11">
-        <f t="shared" si="2"/>
-        <v>0.05</v>
-      </c>
-      <c r="AK5" s="11">
-        <f t="shared" si="2"/>
-        <v>0.05</v>
-      </c>
-      <c r="AL5" s="8">
-        <f t="shared" ref="AL5:AU5" si="7">AK5</f>
-        <v>0.05</v>
-      </c>
-      <c r="AM5" s="8">
-        <f t="shared" si="7"/>
-        <v>0.05</v>
-      </c>
-      <c r="AN5" s="8">
-        <f t="shared" si="7"/>
-        <v>0.05</v>
-      </c>
-      <c r="AO5" s="8">
-        <f t="shared" si="7"/>
-        <v>0.05</v>
-      </c>
-      <c r="AP5" s="8">
-        <f t="shared" si="7"/>
-        <v>0.05</v>
-      </c>
-      <c r="AQ5" s="8">
-        <f t="shared" si="7"/>
-        <v>0.05</v>
-      </c>
-      <c r="AR5" s="8">
-        <f t="shared" si="7"/>
-        <v>0.05</v>
-      </c>
-      <c r="AS5" s="8">
-        <f t="shared" si="7"/>
-        <v>0.05</v>
-      </c>
-      <c r="AT5" s="8">
-        <f t="shared" si="7"/>
-        <v>0.05</v>
-      </c>
-      <c r="AU5" s="8">
-        <f t="shared" si="7"/>
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>36</v>
       </c>
@@ -1605,186 +1194,87 @@
         <v>32</v>
       </c>
       <c r="D6" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="E6" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="F6" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="G6" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="H6" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="I6" s="10" t="b">
-        <f>FALSE()</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" s="10" t="b">
-        <f t="shared" ref="J6:P6" si="8">I6</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" s="10" t="b">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6" s="10" t="b">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M6" s="10" t="b">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N6" s="10" t="b">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" s="10" t="b">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P6" s="10" t="b">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6" s="10" t="b">
-        <f>TRUE()</f>
         <v>1</v>
       </c>
       <c r="R6" s="10" t="b">
-        <f>TRUE()</f>
         <v>1</v>
       </c>
       <c r="S6" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="T6" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="U6" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="V6" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="W6" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="X6" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="Y6" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="Z6" s="10" t="b">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="AA6" s="10" t="b">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="AB6" s="10" t="b">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="AC6" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AD6" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AE6" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AF6" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AG6" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AH6" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AI6" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AJ6" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AK6" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AL6" s="8" t="b">
-        <f t="shared" ref="AL6:AU6" si="9">AK6</f>
-        <v>1</v>
-      </c>
-      <c r="AM6" s="8" t="b">
-        <f t="shared" si="9"/>
-        <v>1</v>
-      </c>
-      <c r="AN6" s="8" t="b">
-        <f t="shared" si="9"/>
-        <v>1</v>
-      </c>
-      <c r="AO6" s="8" t="b">
-        <f t="shared" si="9"/>
-        <v>1</v>
-      </c>
-      <c r="AP6" s="8" t="b">
-        <f t="shared" si="9"/>
-        <v>1</v>
-      </c>
-      <c r="AQ6" s="8" t="b">
-        <f t="shared" si="9"/>
-        <v>1</v>
-      </c>
-      <c r="AR6" s="8" t="b">
-        <f t="shared" si="9"/>
-        <v>1</v>
-      </c>
-      <c r="AS6" s="8" t="b">
-        <f t="shared" si="9"/>
-        <v>1</v>
-      </c>
-      <c r="AT6" s="8" t="b">
-        <f t="shared" si="9"/>
-        <v>1</v>
-      </c>
-      <c r="AU6" s="8" t="b">
-        <f t="shared" si="9"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="str">
-        <f>A6</f>
-        <v>RES_MRGN_10</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>33</v>
@@ -1870,72 +1360,8 @@
       <c r="AC7" s="11">
         <v>0.1</v>
       </c>
-      <c r="AD7" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AE7" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AF7" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AG7" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AH7" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AI7" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AJ7" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AK7" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AL7" s="8">
-        <f t="shared" ref="AL7:AU7" si="10">AK7</f>
-        <v>0.1</v>
-      </c>
-      <c r="AM7" s="8">
-        <f t="shared" si="10"/>
-        <v>0.1</v>
-      </c>
-      <c r="AN7" s="8">
-        <f t="shared" si="10"/>
-        <v>0.1</v>
-      </c>
-      <c r="AO7" s="8">
-        <f t="shared" si="10"/>
-        <v>0.1</v>
-      </c>
-      <c r="AP7" s="8">
-        <f t="shared" si="10"/>
-        <v>0.1</v>
-      </c>
-      <c r="AQ7" s="8">
-        <f t="shared" si="10"/>
-        <v>0.1</v>
-      </c>
-      <c r="AR7" s="8">
-        <f t="shared" si="10"/>
-        <v>0.1</v>
-      </c>
-      <c r="AS7" s="8">
-        <f t="shared" si="10"/>
-        <v>0.1</v>
-      </c>
-      <c r="AT7" s="8">
-        <f t="shared" si="10"/>
-        <v>0.1</v>
-      </c>
-      <c r="AU7" s="8">
-        <f t="shared" si="10"/>
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>37</v>
       </c>
@@ -1946,186 +1372,87 @@
         <v>32</v>
       </c>
       <c r="D8" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="E8" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="F8" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="G8" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="H8" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="I8" s="10" t="b">
-        <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="J8" s="10" t="b">
-        <f t="shared" ref="J8:P8" si="11">I8</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" s="10" t="b">
-        <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" s="10" t="b">
-        <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M8" s="10" t="b">
-        <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N8" s="10" t="b">
-        <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8" s="10" t="b">
-        <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P8" s="10" t="b">
-        <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="10" t="b">
-        <f>FALSE()</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R8" s="10" t="b">
-        <f>TRUE()</f>
         <v>1</v>
       </c>
       <c r="S8" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="T8" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="U8" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="V8" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="W8" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="X8" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="Y8" s="10" t="b">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="Z8" s="10" t="b">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="AA8" s="10" t="b">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="AB8" s="10" t="b">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="AC8" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AD8" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AE8" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AF8" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AG8" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AH8" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AI8" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AJ8" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AK8" s="10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="AL8" s="8" t="b">
-        <f t="shared" ref="AL8:AU8" si="12">AK8</f>
-        <v>1</v>
-      </c>
-      <c r="AM8" s="8" t="b">
-        <f t="shared" si="12"/>
-        <v>1</v>
-      </c>
-      <c r="AN8" s="8" t="b">
-        <f t="shared" si="12"/>
-        <v>1</v>
-      </c>
-      <c r="AO8" s="8" t="b">
-        <f t="shared" si="12"/>
-        <v>1</v>
-      </c>
-      <c r="AP8" s="8" t="b">
-        <f t="shared" si="12"/>
-        <v>1</v>
-      </c>
-      <c r="AQ8" s="8" t="b">
-        <f t="shared" si="12"/>
-        <v>1</v>
-      </c>
-      <c r="AR8" s="8" t="b">
-        <f t="shared" si="12"/>
-        <v>1</v>
-      </c>
-      <c r="AS8" s="8" t="b">
-        <f t="shared" si="12"/>
-        <v>1</v>
-      </c>
-      <c r="AT8" s="8" t="b">
-        <f t="shared" si="12"/>
-        <v>1</v>
-      </c>
-      <c r="AU8" s="8" t="b">
-        <f t="shared" si="12"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="str">
-        <f>A8</f>
-        <v>RES_MRGN_10_31</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>33</v>
@@ -2209,70 +1536,6 @@
         <v>0.1</v>
       </c>
       <c r="AC9" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AD9" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AE9" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AF9" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AG9" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AH9" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AI9" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AJ9" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AK9" s="11">
-        <v>0.1</v>
-      </c>
-      <c r="AL9" s="8">
-        <f t="shared" ref="AL9:AU9" si="13">AK9</f>
-        <v>0.1</v>
-      </c>
-      <c r="AM9" s="8">
-        <f t="shared" si="13"/>
-        <v>0.1</v>
-      </c>
-      <c r="AN9" s="8">
-        <f t="shared" si="13"/>
-        <v>0.1</v>
-      </c>
-      <c r="AO9" s="8">
-        <f t="shared" si="13"/>
-        <v>0.1</v>
-      </c>
-      <c r="AP9" s="8">
-        <f t="shared" si="13"/>
-        <v>0.1</v>
-      </c>
-      <c r="AQ9" s="8">
-        <f t="shared" si="13"/>
-        <v>0.1</v>
-      </c>
-      <c r="AR9" s="8">
-        <f t="shared" si="13"/>
-        <v>0.1</v>
-      </c>
-      <c r="AS9" s="8">
-        <f t="shared" si="13"/>
-        <v>0.1</v>
-      </c>
-      <c r="AT9" s="8">
-        <f t="shared" si="13"/>
-        <v>0.1</v>
-      </c>
-      <c r="AU9" s="8">
-        <f t="shared" si="13"/>
         <v>0.1</v>
       </c>
     </row>
@@ -2283,16 +1546,13 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="AI5 AK5" unlockedFormula="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" customWidth="1"/>
     <col min="2" max="5" width="8.7109375"/>
@@ -2305,7 +1565,7 @@
       <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="22" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="16" t="s">
@@ -2325,10 +1585,10 @@
       <c r="B2" s="12">
         <v>0.25</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="20">
         <v>0.25</v>
       </c>
-      <c r="D2" s="20">
+      <c r="D2" s="21">
         <v>0.25</v>
       </c>
       <c r="E2" s="12">
@@ -2345,10 +1605,10 @@
       <c r="B3" s="13">
         <v>0.5</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="20">
         <v>0.5</v>
       </c>
-      <c r="D3" s="20">
+      <c r="D3" s="21">
         <v>0.5</v>
       </c>
       <c r="E3" s="13">
@@ -2365,10 +1625,10 @@
       <c r="B4" s="12">
         <v>0.5</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="20">
         <v>0.5</v>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="21">
         <v>0.5</v>
       </c>
       <c r="E4" s="12">
@@ -2385,10 +1645,10 @@
       <c r="B5" s="13">
         <v>0.5</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="20">
         <v>0.75</v>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="21">
         <v>0.5</v>
       </c>
       <c r="E5" s="13">
@@ -2405,10 +1665,10 @@
       <c r="B6" s="12">
         <v>1</v>
       </c>
-      <c r="C6" s="12">
-        <v>1</v>
-      </c>
-      <c r="D6" s="20">
+      <c r="C6" s="20">
+        <v>1</v>
+      </c>
+      <c r="D6" s="21">
         <v>1</v>
       </c>
       <c r="E6" s="12">
@@ -2425,10 +1685,10 @@
       <c r="B7" s="13">
         <v>1</v>
       </c>
-      <c r="C7" s="13">
-        <v>1</v>
-      </c>
-      <c r="D7" s="20">
+      <c r="C7" s="20">
+        <v>1</v>
+      </c>
+      <c r="D7" s="21">
         <v>1</v>
       </c>
       <c r="E7" s="13">
@@ -2445,10 +1705,10 @@
       <c r="B8" s="12">
         <v>1</v>
       </c>
-      <c r="C8" s="12">
-        <v>1</v>
-      </c>
-      <c r="D8" s="20">
+      <c r="C8" s="20">
+        <v>1</v>
+      </c>
+      <c r="D8" s="21">
         <v>1</v>
       </c>
       <c r="E8" s="12">
@@ -2465,10 +1725,10 @@
       <c r="B9" s="13">
         <v>1</v>
       </c>
-      <c r="C9" s="13">
-        <v>1</v>
-      </c>
-      <c r="D9" s="20">
+      <c r="C9" s="20">
+        <v>1</v>
+      </c>
+      <c r="D9" s="21">
         <v>1</v>
       </c>
       <c r="E9" s="13">
@@ -2485,10 +1745,10 @@
       <c r="B10" s="12">
         <v>0.53</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="20">
         <v>0.53</v>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="21">
         <v>1</v>
       </c>
       <c r="E10" s="12">
@@ -2505,10 +1765,10 @@
       <c r="B11" s="13">
         <v>1</v>
       </c>
-      <c r="C11" s="13">
-        <v>1</v>
-      </c>
-      <c r="D11" s="20">
+      <c r="C11" s="20">
+        <v>1</v>
+      </c>
+      <c r="D11" s="21">
         <v>1</v>
       </c>
       <c r="E11" s="13">
@@ -2525,10 +1785,10 @@
       <c r="B12" s="12">
         <v>1</v>
       </c>
-      <c r="C12" s="12">
-        <v>1</v>
-      </c>
-      <c r="D12" s="20">
+      <c r="C12" s="20">
+        <v>1</v>
+      </c>
+      <c r="D12" s="21">
         <v>1</v>
       </c>
       <c r="E12" s="12">
@@ -2545,10 +1805,10 @@
       <c r="B13" s="13">
         <v>1</v>
       </c>
-      <c r="C13" s="13">
-        <v>1</v>
-      </c>
-      <c r="D13" s="20">
+      <c r="C13" s="20">
+        <v>1</v>
+      </c>
+      <c r="D13" s="21">
         <v>1</v>
       </c>
       <c r="E13" s="13">
@@ -2565,10 +1825,10 @@
       <c r="B14" s="12">
         <v>1</v>
       </c>
-      <c r="C14" s="12">
-        <v>1</v>
-      </c>
-      <c r="D14" s="20">
+      <c r="C14" s="20">
+        <v>1</v>
+      </c>
+      <c r="D14" s="21">
         <v>1</v>
       </c>
       <c r="E14" s="12">
@@ -2585,10 +1845,10 @@
       <c r="B15" s="13">
         <v>1</v>
       </c>
-      <c r="C15" s="13">
-        <v>1</v>
-      </c>
-      <c r="D15" s="20">
+      <c r="C15" s="20">
+        <v>1</v>
+      </c>
+      <c r="D15" s="21">
         <v>1</v>
       </c>
       <c r="E15" s="13">
@@ -2605,10 +1865,10 @@
       <c r="B16" s="12">
         <v>1</v>
       </c>
-      <c r="C16" s="12">
-        <v>1</v>
-      </c>
-      <c r="D16" s="20">
+      <c r="C16" s="20">
+        <v>1</v>
+      </c>
+      <c r="D16" s="21">
         <v>1</v>
       </c>
       <c r="E16" s="12">
@@ -2625,10 +1885,10 @@
       <c r="B17" s="13">
         <v>1</v>
       </c>
-      <c r="C17" s="13">
-        <v>1</v>
-      </c>
-      <c r="D17" s="20">
+      <c r="C17" s="20">
+        <v>1</v>
+      </c>
+      <c r="D17" s="21">
         <v>1</v>
       </c>
       <c r="E17" s="13">
@@ -2645,10 +1905,10 @@
       <c r="B18" s="12">
         <v>1</v>
       </c>
-      <c r="C18" s="12">
-        <v>1</v>
-      </c>
-      <c r="D18" s="20">
+      <c r="C18" s="20">
+        <v>1</v>
+      </c>
+      <c r="D18" s="21">
         <v>1</v>
       </c>
       <c r="E18" s="12">
@@ -2665,10 +1925,10 @@
       <c r="B19" s="13">
         <v>1</v>
       </c>
-      <c r="C19" s="13">
-        <v>1</v>
-      </c>
-      <c r="D19" s="20">
+      <c r="C19" s="20">
+        <v>1</v>
+      </c>
+      <c r="D19" s="21">
         <v>1</v>
       </c>
       <c r="E19" s="13">
@@ -2685,10 +1945,10 @@
       <c r="B20" s="12">
         <v>0</v>
       </c>
-      <c r="C20" s="12">
-        <v>0</v>
-      </c>
-      <c r="D20" s="20">
+      <c r="C20" s="20">
+        <v>0</v>
+      </c>
+      <c r="D20" s="21">
         <v>0</v>
       </c>
       <c r="E20" s="12">
@@ -2705,10 +1965,10 @@
       <c r="B21" s="13">
         <v>0</v>
       </c>
-      <c r="C21" s="13">
-        <v>0</v>
-      </c>
-      <c r="D21" s="20">
+      <c r="C21" s="20">
+        <v>0</v>
+      </c>
+      <c r="D21" s="21">
         <v>0</v>
       </c>
       <c r="E21" s="13">
@@ -2725,10 +1985,10 @@
       <c r="B22" s="12">
         <v>0</v>
       </c>
-      <c r="C22" s="12">
-        <v>0</v>
-      </c>
-      <c r="D22" s="20">
+      <c r="C22" s="20">
+        <v>0</v>
+      </c>
+      <c r="D22" s="21">
         <v>0</v>
       </c>
       <c r="E22" s="12">
@@ -2745,10 +2005,10 @@
       <c r="B23" s="13">
         <v>0.5</v>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="20">
         <v>0.5</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="21">
         <v>0.5</v>
       </c>
       <c r="E23" s="13">
@@ -2765,10 +2025,10 @@
       <c r="B24" s="12">
         <v>0.1</v>
       </c>
-      <c r="C24" s="12">
-        <v>0.1</v>
-      </c>
-      <c r="D24" s="20">
+      <c r="C24" s="20">
+        <v>0.1</v>
+      </c>
+      <c r="D24" s="21">
         <v>0.1</v>
       </c>
       <c r="E24" s="12">
@@ -2785,10 +2045,10 @@
       <c r="B25" s="13">
         <v>0.1</v>
       </c>
-      <c r="C25" s="13">
-        <v>0.1</v>
-      </c>
-      <c r="D25" s="20">
+      <c r="C25" s="20">
+        <v>0.1</v>
+      </c>
+      <c r="D25" s="21">
         <v>0.1</v>
       </c>
       <c r="E25" s="13">

</xml_diff>